<commit_message>
READ ME: full how-to-read guides for the buyer/seller margin and ADX
Omar 2026-07-28: the WHAT THE NUMBERS MEAN section now carries the plain
reading scales - margin (+15 buyers in charge / single digits nobody owns /
zero stalemate / negative blocked, plus the measured no-edge caveat) and
ADX (never read as a percent: <20 chop, 20-25 forming, 25-40 real where 35
is strong, 40-60 late, 60+ rare; strength not direction; slow, confirming).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-28_new.xlsx
+++ b/reports/universe_2026-07-28_new.xlsx
@@ -1580,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28 16:35 local</t>
+          <t>2026-07-28 18:23 local</t>
         </is>
       </c>
     </row>
@@ -2059,89 +2059,101 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Buying pressure minus selling pressure (+DI - -DI). Who is winning the daily fight. MEASURED 2026-07-28: across 170 signals it did NOT predict returns (slightly backwards), so it is context only - never a rank, never a veto.</t>
+          <t>Buying pressure minus selling pressure over the last 14 days - the scoreboard of the daily tug-of-war. HOW TO READ IT: +15 or more = buyers clearly in charge (SJM was +18 the day it was bought). Low single digits = buyers barely ahead - the trend looks strong but nobody really owns it (MLI's +4 tell). Near zero = stalemate, a yellow flag on a fresh buy. Negative on a buy signal = sellers still winning; the gates block these. CAVEAT, measured 2026-07-28 on 170 signals: a big margin did NOT predict better returns (slightly backwards). Read it like a fuel gauge, not a map: it describes the current state of who controls the stock - never a reason by itself to buy, rank higher, or pay up.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Trend Strength vs Today's Best</t>
+          <t>Trend Strength (ADX)</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Each name's ADX as a share of the day's strongest (100 = strongest today). Trend strength is the one measured-to-matter input, so this ranks the batch by it at a glance.</t>
+          <t>Technically a 0-100 scale but real readings almost never get near 100, so do NOT read it as a percent. HOW TO READ IT: below 20 = no trend, sideways chop (our gates require 20+). 20-25 = a trend is forming. 25-40 = a genuine, tradeable trend - most good entries live here; 35 is STRONG, not mediocre. 40-60 = powerful and often late. 60+ = rare (panics and parabolas). It measures strength only, not direction - a crash reads high too. And it is SLOW (built from smoothed 14-day averages): it confirms a trend that exists, it does not predict one. A gate and a ranking aid, never a buy signal by itself.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Magical (CCI-20)</t>
+          <t>Trend Strength vs Today's Best</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Above +100 = overbought, below -100 = oversold. NOTE: measured 2026-07-22 across 1,725 signals, this cut does NOT separate returns (0.03pt over 21 days). Treat as context, not a veto.</t>
+          <t>Each name's ADX as a share of the day's strongest (100 = strongest today). Fixes the read-as-percent trap above: a 35 that is today's best reads 100. Trend strength is the one measured-to-matter input, so this ranks the batch by it at a glance.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>ZLSMA-50</t>
+          <t>Magical (CCI-20)</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>The trend line. Price below it on a buy signal is a structural fail.</t>
+          <t>Above +100 = overbought, below -100 = oversold. NOTE: measured 2026-07-22 across 1,725 signals, this cut does NOT separate returns (0.03pt over 21 days). Treat as context, not a veto.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Chandelier Exit</t>
+          <t>ZLSMA-50</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Flips BUY/SELL. The label price is the STOP level, not an entry.</t>
+          <t>The trend line. Price below it on a buy signal is a structural fail.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Regime PASS</t>
+          <t>Chandelier Exit</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Above a rising 200-day and beating SPY -&gt; normal size.</t>
+          <t>Flips BUY/SELL. The label price is the STOP level, not an entry.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
+          <t>Regime PASS</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Above a rising 200-day and beating SPY -&gt; normal size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
           <t>Regime REPAIR</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>Below the 200-day -&gt; starter size only.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="7" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>Regime DEEP-FAIL</t>
         </is>
       </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>More than 10% below the 200-day -&gt; watch only, no size.</t>
         </is>
@@ -26174,7 +26186,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>2026-07-28 16:35 local</t>
+          <t>2026-07-28 18:23 local</t>
         </is>
       </c>
     </row>
@@ -28654,7 +28666,7 @@
         <v>65.09999999999999</v>
       </c>
       <c r="Q4" s="23" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
       <c r="R4" s="20" t="n">
         <v>97</v>
@@ -28747,7 +28759,7 @@
         <v>58.2</v>
       </c>
       <c r="Q5" s="23" t="n">
-        <v>1.04</v>
+        <v>1.21</v>
       </c>
       <c r="R5" s="20" t="n">
         <v>97.40000000000001</v>
@@ -28848,7 +28860,7 @@
         <v>62.8</v>
       </c>
       <c r="Q6" s="23" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="R6" s="20" t="n">
         <v>97.59999999999999</v>
@@ -29121,7 +29133,7 @@
         <v>54.2</v>
       </c>
       <c r="Q9" s="23" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="R9" s="20" t="n">
         <v>85</v>
@@ -29214,7 +29226,7 @@
         <v>64.3</v>
       </c>
       <c r="Q10" s="23" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="R10" s="20" t="n">
         <v>95</v>
@@ -29394,7 +29406,7 @@
         <v>61.3</v>
       </c>
       <c r="Q12" s="23" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="R12" s="20" t="n">
         <v>97.7</v>
@@ -29861,7 +29873,7 @@
         <v>59.5</v>
       </c>
       <c r="Q17" s="23" t="n">
-        <v>1.14</v>
+        <v>1.15</v>
       </c>
       <c r="R17" s="20" t="n">
         <v>93.40000000000001</v>
@@ -29954,7 +29966,7 @@
         <v>56.5</v>
       </c>
       <c r="Q18" s="23" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="R18" s="20" t="n">
         <v>83.3</v>
@@ -30237,7 +30249,7 @@
         <v>73.7</v>
       </c>
       <c r="Q21" s="30" t="n">
-        <v>1.64</v>
+        <v>1.65</v>
       </c>
       <c r="R21" s="27" t="n">
         <v>99.09999999999999</v>
@@ -30518,7 +30530,7 @@
         <v>65.7</v>
       </c>
       <c r="Q24" s="30" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="R24" s="27" t="n">
         <v>57.5</v>
@@ -30605,7 +30617,7 @@
         <v>62.6</v>
       </c>
       <c r="Q25" s="30" t="n">
-        <v>1.4</v>
+        <v>1.42</v>
       </c>
       <c r="R25" s="27" t="n">
         <v>84.09999999999999</v>
@@ -30700,7 +30712,7 @@
         <v>61.9</v>
       </c>
       <c r="Q26" s="30" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="R26" s="27" t="n">
         <v>61.2</v>
@@ -31141,7 +31153,7 @@
         <v>64.7</v>
       </c>
       <c r="Q31" s="30" t="n">
-        <v>1.89</v>
+        <v>2.1</v>
       </c>
       <c r="R31" s="27" t="n">
         <v>81.7</v>
@@ -31483,7 +31495,7 @@
         <v>61.1</v>
       </c>
       <c r="Q35" s="30" t="n">
-        <v>0.8</v>
+        <v>0.97</v>
       </c>
       <c r="R35" s="27" t="n">
         <v>93.2</v>
@@ -31570,7 +31582,7 @@
         <v>58.1</v>
       </c>
       <c r="Q36" s="30" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="R36" s="27" t="n">
         <v>93.3</v>
@@ -31758,7 +31770,7 @@
         <v>61.3</v>
       </c>
       <c r="Q38" s="30" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
       <c r="R38" s="27" t="n">
         <v>77.2</v>
@@ -31853,7 +31865,7 @@
         <v>56.8</v>
       </c>
       <c r="Q39" s="30" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="R39" s="27" t="n">
         <v>63.7</v>
@@ -32035,7 +32047,7 @@
         <v>58.5</v>
       </c>
       <c r="Q41" s="30" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="R41" s="27" t="n">
         <v>96.90000000000001</v>
@@ -32215,7 +32227,7 @@
         <v>55.7</v>
       </c>
       <c r="Q43" s="30" t="n">
-        <v>1.09</v>
+        <v>1.16</v>
       </c>
       <c r="R43" s="27" t="n">
         <v>74.5</v>
@@ -32302,7 +32314,7 @@
         <v>51.6</v>
       </c>
       <c r="Q44" s="30" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="R44" s="27" t="n">
         <v>79.90000000000001</v>
@@ -32476,7 +32488,7 @@
         <v>67.5</v>
       </c>
       <c r="Q46" s="30" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="R46" s="27" t="n">
         <v>99.40000000000001</v>
@@ -32753,7 +32765,7 @@
         <v>48.5</v>
       </c>
       <c r="Q49" s="30" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="R49" s="27" t="n">
         <v>85.3</v>
@@ -33034,7 +33046,7 @@
         <v>54.3</v>
       </c>
       <c r="Q52" s="30" t="n">
-        <v>1.46</v>
+        <v>1.47</v>
       </c>
       <c r="R52" s="27" t="n">
         <v>52</v>
@@ -33570,7 +33582,7 @@
         <v>47.9</v>
       </c>
       <c r="Q58" s="30" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
       <c r="R58" s="27" t="n">
         <v>35.8</v>
@@ -33825,7 +33837,7 @@
         <v>56.2</v>
       </c>
       <c r="Q61" s="30" t="n">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
       <c r="R61" s="27" t="n">
         <v>90.8</v>
@@ -34098,7 +34110,7 @@
         <v>56.7</v>
       </c>
       <c r="Q64" s="30" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="R64" s="27" t="n">
         <v>93.7</v>
@@ -34371,7 +34383,7 @@
         <v>54.1</v>
       </c>
       <c r="Q67" s="30" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="R67" s="27" t="n">
         <v>97.40000000000001</v>
@@ -34646,7 +34658,7 @@
         <v>48</v>
       </c>
       <c r="Q70" s="30" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R70" s="27" t="n">
         <v>45.6</v>
@@ -34982,7 +34994,7 @@
         <v>57</v>
       </c>
       <c r="Q74" s="30" t="n">
-        <v>1.43</v>
+        <v>1.44</v>
       </c>
       <c r="R74" s="27" t="n">
         <v>61.8</v>

</xml_diff>

<commit_message>
Track Record: TOP SKIPPED RUNNERS block under MY TRADES
Top 10 unactioned still-open picks ranked by run since the earliest open
recommendation, one row per ticker, actioned names excluded - the
pre-sorted missed-money leaderboard Omar asked for, and the raw material
for the selection-vs-pool test. side_table gains a start_row param so
blocks can stack.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/universe_2026-07-28_new.xlsx
+++ b/reports/universe_2026-07-28_new.xlsx
@@ -545,6 +545,48 @@
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>The same, as a percent of entry.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="N10" authorId="0" shapeId="0">
+      <text>
+        <t>Recommendations Omar did NOT act on, ranked by how far they have run since the earliest still-open pick. The honest missed-money scorecard: it exists so skips get graded, not to feel good. Compare against MY TRADES above - that comparison is the test of whether hand-picking beats the pool it picks from.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="O10" authorId="0" shapeId="0">
+      <text>
+        <t>The earliest open recommendation date.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="P10" authorId="0" shapeId="0">
+      <text>
+        <t>Price on the pick date.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="Q10" authorId="0" shapeId="0">
+      <text>
+        <t>Latest tracked price.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="R10" authorId="0" shapeId="0">
+      <text>
+        <t>The run that was skipped.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="S10" authorId="0" shapeId="0">
+      <text>
+        <t>Best point reached since the pick.
+(Full guide: 'READ ME FIRST' tab)</t>
+      </text>
+    </comment>
+    <comment ref="T10" authorId="0" shapeId="0">
+      <text>
+        <t>Days since the pick.
 (Full guide: 'READ ME FIRST' tab)</t>
       </text>
     </comment>
@@ -1622,7 +1664,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-07-28 18:37 local</t>
+          <t>2026-07-28 19:19 local</t>
         </is>
       </c>
     </row>
@@ -2432,14 +2474,14 @@
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="9" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -3106,6 +3148,41 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N10" s="29" t="inlineStr">
+        <is>
+          <t>TOP SKIPPED RUNNERS</t>
+        </is>
+      </c>
+      <c r="O10" s="29" t="inlineStr">
+        <is>
+          <t>Picked On</t>
+        </is>
+      </c>
+      <c r="P10" s="29" t="inlineStr">
+        <is>
+          <t>Price Then</t>
+        </is>
+      </c>
+      <c r="Q10" s="29" t="inlineStr">
+        <is>
+          <t>Price Now</t>
+        </is>
+      </c>
+      <c r="R10" s="29" t="inlineStr">
+        <is>
+          <t>% Since</t>
+        </is>
+      </c>
+      <c r="S10" s="29" t="inlineStr">
+        <is>
+          <t>Best %</t>
+        </is>
+      </c>
+      <c r="T10" s="29" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="33" t="inlineStr">
@@ -3152,6 +3229,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N11" s="45" t="inlineStr">
+        <is>
+          <t>PBF</t>
+        </is>
+      </c>
+      <c r="O11" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="P11" s="48" t="n">
+        <v>48.04</v>
+      </c>
+      <c r="Q11" s="48" t="n">
+        <v>61</v>
+      </c>
+      <c r="R11" s="49" t="n">
+        <v>27.59</v>
+      </c>
+      <c r="S11" s="49" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="T11" s="47" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="33" t="inlineStr">
@@ -3198,6 +3300,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N12" s="45" t="inlineStr">
+        <is>
+          <t>CDNA</t>
+        </is>
+      </c>
+      <c r="O12" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="P12" s="48" t="n">
+        <v>29.06</v>
+      </c>
+      <c r="Q12" s="48" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="R12" s="49" t="n">
+        <v>26.28</v>
+      </c>
+      <c r="S12" s="49" t="n">
+        <v>43</v>
+      </c>
+      <c r="T12" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="33" t="inlineStr">
@@ -3244,6 +3371,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N13" s="45" t="inlineStr">
+        <is>
+          <t>TXG</t>
+        </is>
+      </c>
+      <c r="O13" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="P13" s="48" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q13" s="48" t="n">
+        <v>47.05</v>
+      </c>
+      <c r="R13" s="49" t="n">
+        <v>24.37</v>
+      </c>
+      <c r="S13" s="49" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="T13" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="33" t="inlineStr">
@@ -3290,6 +3442,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N14" s="45" t="inlineStr">
+        <is>
+          <t>ETON</t>
+        </is>
+      </c>
+      <c r="O14" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="P14" s="48" t="n">
+        <v>38.02</v>
+      </c>
+      <c r="Q14" s="48" t="n">
+        <v>46.66</v>
+      </c>
+      <c r="R14" s="49" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="S14" s="49" t="n">
+        <v>25</v>
+      </c>
+      <c r="T14" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="33" t="inlineStr">
@@ -3336,6 +3513,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N15" s="45" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="O15" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="P15" s="48" t="n">
+        <v>53.14</v>
+      </c>
+      <c r="Q15" s="48" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="R15" s="49" t="n">
+        <v>19.37</v>
+      </c>
+      <c r="S15" s="49" t="n">
+        <v>31</v>
+      </c>
+      <c r="T15" s="47" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="33" t="inlineStr">
@@ -3382,6 +3584,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N16" s="45" t="inlineStr">
+        <is>
+          <t>FTRE</t>
+        </is>
+      </c>
+      <c r="O16" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="P16" s="48" t="n">
+        <v>17.85</v>
+      </c>
+      <c r="Q16" s="48" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="R16" s="49" t="n">
+        <v>18.42</v>
+      </c>
+      <c r="S16" s="49" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="T16" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="33" t="inlineStr">
@@ -3428,6 +3655,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N17" s="45" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+      <c r="O17" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="P17" s="48" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="Q17" s="48" t="n">
+        <v>89.31</v>
+      </c>
+      <c r="R17" s="49" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="S17" s="49" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="T17" s="47" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="33" t="inlineStr">
@@ -3478,6 +3730,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N18" s="45" t="inlineStr">
+        <is>
+          <t>CAKE</t>
+        </is>
+      </c>
+      <c r="O18" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="P18" s="48" t="n">
+        <v>76.89</v>
+      </c>
+      <c r="Q18" s="48" t="n">
+        <v>89.01000000000001</v>
+      </c>
+      <c r="R18" s="49" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="S18" s="49" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="T18" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="23" t="inlineStr">
@@ -3528,6 +3805,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N19" s="45" t="inlineStr">
+        <is>
+          <t>BJRI</t>
+        </is>
+      </c>
+      <c r="O19" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="P19" s="48" t="n">
+        <v>59.19</v>
+      </c>
+      <c r="Q19" s="48" t="n">
+        <v>68.95</v>
+      </c>
+      <c r="R19" s="49" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="S19" s="49" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="T19" s="47" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="56" t="inlineStr">
@@ -3578,6 +3880,31 @@
           <t>OPEN</t>
         </is>
       </c>
+      <c r="N20" s="45" t="inlineStr">
+        <is>
+          <t>WKC</t>
+        </is>
+      </c>
+      <c r="O20" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P20" s="48" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="Q20" s="48" t="n">
+        <v>40.05</v>
+      </c>
+      <c r="R20" s="49" t="n">
+        <v>13.39</v>
+      </c>
+      <c r="S20" s="49" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="T20" s="47" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="33" t="inlineStr">
@@ -3626,6 +3953,11 @@
       <c r="L21" s="35" t="inlineStr">
         <is>
           <t>OPEN</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Top 10 of 339 skipped open picks. A skip that ran is a graded miss, not a non-event - and a skip that fell is risk avoided. Both belong on the Friday scorecard.</t>
         </is>
       </c>
     </row>
@@ -26165,7 +26497,7 @@
       </c>
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>2026-07-28 18:37 local</t>
+          <t>2026-07-28 19:19 local</t>
         </is>
       </c>
     </row>
@@ -30521,7 +30853,7 @@
         <v>62.6</v>
       </c>
       <c r="Q25" s="28" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
       <c r="R25" s="26" t="n">
         <v>84.09999999999999</v>
@@ -33303,7 +33635,7 @@
         <v>68.3</v>
       </c>
       <c r="Q57" s="28" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="R57" s="26" t="n">
         <v>65.09999999999999</v>

</xml_diff>